<commit_message>
Aggiunge Spyro, due membri placeholder e aggiorna documenti/membri da Excel
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/membri_gilda.xlsx
+++ b/membri_gilda.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sielte-my.sharepoint.com/personal/a_guidetti_sielte_it/Documents/Documenti Personali/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\central_ai\gilda-dei-matti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="121" documentId="8_{6BAE6E0C-F9E5-4CD1-A905-49BB89FE3E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0B61241-52BD-4D44-9E85-B466F4C53F20}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B2F7DD-1552-42E8-925E-620D33230E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4380" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Membri" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="75">
   <si>
     <t>Nome Personaggio</t>
   </si>
@@ -106,9 +106,6 @@
     <t>Selune</t>
   </si>
   <si>
-    <t>Gabbro è nato a Pozzak. Famoso per le sue doti di navigatore, ha conosce perfettamente tutte le rive del Lago Brodom. Il suo carattere vivace e simpatico gli ha permesso di farsi numerosi amici in diverse città. Viaggia accompagnato dal suo Clarinetto, con cui suona armoniose melodie e colpisce con violenza i nemici. La sua natura di Bullywug gli ha permesso di sviluppare una grande conoscenza dei veleni e delle sostanze tossiche.</t>
-  </si>
-  <si>
     <t>150 mo</t>
   </si>
   <si>
@@ -215,6 +212,45 @@
   </si>
   <si>
     <t>Legale Buono</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrik è il classico inventore pazzo. Per anni ha servito Giorgione in cucina ed è diventato la sua spalla, assecondando tutte le sue bizzarre richieste. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una gnoma calma e molto intelligente, predilige le invenzioni che possono supportare i suoi amici. </t>
+  </si>
+  <si>
+    <t>Beatrice Kiddo, tiefling infernale e stregona di talento, nacque sotto una rara congiunzione astrale che, a detta degli astrologi, prometteva grandi poteri e una vita fuori dall’ordinario. Gli astrologi avevano ragione… anche se probabilmente non immaginavano esattamente quanto fuori dall’ordinario. Per ben 69 anni, Beatrice visse una vita di agi, sete pregiate, gioielli scintillanti e lenzuola di seta. Dotata di un fascino quasi soprannaturale e di una magia innata capace di incantare chiunque la incontrasse, sfruttò le proprie doti per frequentare nobili, mercanti, ufficiali e ogni genere di uomo disposto a riempirle le tasche e non solo… in cambio della sua compagnia. Mentre altri stregoni passavano il tempo a studiare antichi tomi o a combattere mostri, Beatrice perfezionava arti decisamente più redditizie. Con il passare dei decenni, però, la vita dorata iniziò a sembrarle monotona e si pose una domanda sconvolgente:</t>
+  </si>
+  <si>
+    <t>“E se provassi qualcosa di diverso?”</t>
+  </si>
+  <si>
+    <t>Fu così che decise di diventare un’avventuriera,ma certe abitudini sono dure a morire.</t>
+  </si>
+  <si>
+    <t>Spyro</t>
+  </si>
+  <si>
+    <t>Dragonide</t>
+  </si>
+  <si>
+    <t>Caotico Buono</t>
+  </si>
+  <si>
+    <t>Nuovo</t>
+  </si>
+  <si>
+    <t>Cresciuto nella bottega di gemme del padre, ha imparato l’arte della contrattazione prima ancora di saper leggere. Dopo il fallimento dell'attività a causa della malattia del genitore, è sceso negli oscuri vicoli cittadini per sopravvivere. Trasformando il suo ingegno in astuzia, ha imparato a scassinare serrature e a manipolare la realtà tramite l’illusione, usando l’inganno come unico scudo contro la miseria. Ora viaggia portando con sé solo le sue erbe, un bastone magico e lo sguardo cinico di chi sa che, in questo mondo, tutto ha un prezzo.</t>
+  </si>
+  <si>
+    <t>Dalila</t>
+  </si>
+  <si>
+    <t>Giuseppe</t>
+  </si>
+  <si>
+    <t>placeholder</t>
   </si>
 </sst>
 </file>
@@ -264,7 +300,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -300,11 +336,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -331,6 +382,19 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -633,7 +697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -684,18 +748,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" s="4" customFormat="1" ht="242.25" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="C2" s="2">
         <v>5</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>23</v>
@@ -705,24 +769,28 @@
       <c r="H2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="J2" s="3">
+        <v>116</v>
+      </c>
       <c r="K2" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C3" s="2">
         <v>5</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>23</v>
@@ -733,23 +801,25 @@
         <v>17</v>
       </c>
       <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
+      <c r="J3" s="3">
+        <v>47</v>
+      </c>
       <c r="K3" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>49</v>
       </c>
       <c r="C4" s="2">
         <v>5</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>23</v>
@@ -759,18 +829,22 @@
       <c r="H4" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="I4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="J4" s="3">
+        <v>36</v>
+      </c>
       <c r="K4" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>41</v>
       </c>
       <c r="C5" s="2">
         <v>5</v>
@@ -789,10 +863,10 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" s="4" customFormat="1" ht="114.75" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>20</v>
       </c>
@@ -818,18 +892,18 @@
         <v>17</v>
       </c>
       <c r="I6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="K6" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>12</v>
@@ -838,7 +912,7 @@
         <v>4</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>23</v>
@@ -851,22 +925,22 @@
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2">
         <v>1</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>36</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>37</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -883,10 +957,10 @@
     </row>
     <row r="9" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>32</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>33</v>
       </c>
       <c r="C9" s="2">
         <v>6</v>
@@ -895,7 +969,7 @@
         <v>13</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="7" t="s">
@@ -914,16 +988,16 @@
     </row>
     <row r="10" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>30</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>23</v>
@@ -934,9 +1008,11 @@
         <v>17</v>
       </c>
       <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
+      <c r="J10" s="3">
+        <v>80</v>
+      </c>
       <c r="K10" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:11" s="4" customFormat="1" ht="229.5" x14ac:dyDescent="0.25">
@@ -974,24 +1050,24 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="51" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>57</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>58</v>
       </c>
       <c r="C12" s="7">
         <v>3</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E12" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>59</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>60</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>16</v>
@@ -999,7 +1075,9 @@
       <c r="H12" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="8"/>
+      <c r="I12" s="8" t="s">
+        <v>62</v>
+      </c>
       <c r="J12" s="8" t="s">
         <v>16</v>
       </c>
@@ -1007,24 +1085,24 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C13" s="7">
         <v>3</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>16</v>
@@ -1032,7 +1110,9 @@
       <c r="H13" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I13" s="8"/>
+      <c r="I13" s="8" t="s">
+        <v>63</v>
+      </c>
       <c r="J13" s="8" t="s">
         <v>16</v>
       </c>
@@ -1040,18 +1120,77 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
+    <row r="14" spans="1:11" ht="180" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="10">
+        <v>3</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="J14" s="12">
+        <v>78</v>
+      </c>
+      <c r="K14" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{00000000-0001-0000-0000-000000000000}">

</xml_diff>

<commit_message>
Membri: aggiunge Occhio di Falco
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/membri_gilda.xlsx
+++ b/membri_gilda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\central_ai\gilda-dei-matti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B2F7DD-1552-42E8-925E-620D33230E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D10EAA1A-E613-4195-B728-2FC0B5DE37C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="79">
   <si>
     <t>Nome Personaggio</t>
   </si>
@@ -251,6 +251,18 @@
   </si>
   <si>
     <t>placeholder</t>
+  </si>
+  <si>
+    <t>Occhio di Falco</t>
+  </si>
+  <si>
+    <t>Elfo Alto</t>
+  </si>
+  <si>
+    <t>Neutrale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La mia famiglia abitava nel bosco in un territorio ostile, mi hanno insegnato l'arte di cacciare fin da ragazza, per proteggere il nostro clan. Dovendo dormire solo 4 ore a notte però ho fatto amicizia con molti animali, miei unici compagni. </t>
   </si>
 </sst>
 </file>
@@ -391,10 +403,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1159,38 +1171,70 @@
       <c r="A15" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13"/>
+    </row>
+    <row r="17" spans="1:11" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="10">
+        <v>3</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="J17" s="13">
+        <v>10</v>
+      </c>
+      <c r="K17" s="12" t="s">
+        <v>53</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{00000000-0001-0000-0000-000000000000}">
@@ -1204,6 +1248,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_activity xmlns="b29cbc76-272b-40e5-b4ba-3e4af727d16b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100335EAE044E422D4BAEC0B1BC71186902" ma:contentTypeVersion="20" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="8191542849a603e5cc73d892766c41f0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns3="b29cbc76-272b-40e5-b4ba-3e4af727d16b" xmlns:ns4="abdbd0a1-ed93-4afe-bb88-a490c0734ad3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cc47de22a57756af56b6fd27515aad7d" ns1:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1473,41 +1536,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_activity xmlns="b29cbc76-272b-40e5-b4ba-3e4af727d16b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E71A66E7-14C5-4436-B338-E9FE6616C4F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{702E6FB5-6A67-4034-9986-FD37F4044FFB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="b29cbc76-272b-40e5-b4ba-3e4af727d16b"/>
-    <ds:schemaRef ds:uri="abdbd0a1-ed93-4afe-bb88-a490c0734ad3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1531,9 +1563,21 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{702E6FB5-6A67-4034-9986-FD37F4044FFB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E71A66E7-14C5-4436-B338-E9FE6616C4F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="b29cbc76-272b-40e5-b4ba-3e4af727d16b"/>
+    <ds:schemaRef ds:uri="abdbd0a1-ed93-4afe-bb88-a490c0734ad3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Membri: aggiorna descrizioni dei personaggi
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/membri_gilda.xlsx
+++ b/membri_gilda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\central_ai\gilda-dei-matti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D10EAA1A-E613-4195-B728-2FC0B5DE37C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5F5B64-024B-47DB-9A9C-B816630A6E2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="82">
   <si>
     <t>Nome Personaggio</t>
   </si>
@@ -220,15 +220,6 @@
     <t xml:space="preserve">Una gnoma calma e molto intelligente, predilige le invenzioni che possono supportare i suoi amici. </t>
   </si>
   <si>
-    <t>Beatrice Kiddo, tiefling infernale e stregona di talento, nacque sotto una rara congiunzione astrale che, a detta degli astrologi, prometteva grandi poteri e una vita fuori dall’ordinario. Gli astrologi avevano ragione… anche se probabilmente non immaginavano esattamente quanto fuori dall’ordinario. Per ben 69 anni, Beatrice visse una vita di agi, sete pregiate, gioielli scintillanti e lenzuola di seta. Dotata di un fascino quasi soprannaturale e di una magia innata capace di incantare chiunque la incontrasse, sfruttò le proprie doti per frequentare nobili, mercanti, ufficiali e ogni genere di uomo disposto a riempirle le tasche e non solo… in cambio della sua compagnia. Mentre altri stregoni passavano il tempo a studiare antichi tomi o a combattere mostri, Beatrice perfezionava arti decisamente più redditizie. Con il passare dei decenni, però, la vita dorata iniziò a sembrarle monotona e si pose una domanda sconvolgente:</t>
-  </si>
-  <si>
-    <t>“E se provassi qualcosa di diverso?”</t>
-  </si>
-  <si>
-    <t>Fu così che decise di diventare un’avventuriera,ma certe abitudini sono dure a morire.</t>
-  </si>
-  <si>
     <t>Spyro</t>
   </si>
   <si>
@@ -263,6 +254,24 @@
   </si>
   <si>
     <t xml:space="preserve">La mia famiglia abitava nel bosco in un territorio ostile, mi hanno insegnato l'arte di cacciare fin da ragazza, per proteggere il nostro clan. Dovendo dormire solo 4 ore a notte però ho fatto amicizia con molti animali, miei unici compagni. </t>
+  </si>
+  <si>
+    <t>Beatrice Kiddo, tiefling infernale e stregona di talento, nacque sotto una rara congiunzione astrale che, a detta degli astrologi, prometteva grandi poteri e una vita fuori dall’ordinario. Gli astrologi avevano ragione… anche se probabilmente non immaginavano esattamente quanto fuori dall’ordinario. Per ben 69 anni, Beatrice visse una vita di agi, sete pregiate, gioielli scintillanti e lenzuola di seta. Dotata di un fascino quasi soprannaturale e di una magia innata capace di incantare chiunque la incontrasse, sfruttò le proprie doti per frequentare nobili, mercanti, ufficiali e ogni genere di uomo disposto a riempirle le tasche e non solo… in cambio della sua compagnia. Mentre altri stregoni passavano il tempo a studiare antichi tomi o a combattere mostri, Beatrice perfezionava arti decisamente più redditizie. Con il passare dei decenni, però, la vita dorata iniziò a sembrarle monotona e si pose una domanda sconvolgente:“E se provassi qualcosa di diverso?” Fu così che decise di diventare un’avventuriera,ma certe abitudini sono dure a morire.</t>
+  </si>
+  <si>
+    <t>Nata con una curiosità insaziabile, è stata assunta come apprendista da un potente mago, il cui compito principale era tuttavia quello di fare da "baby-sitter" ai suoi turbolenti nipoti. Tra un incantesimo di pulizia e il recupero di bambini fluttuanti per la torre, ha imparato più magia pratica in un pomeriggio che leggendo tomi polverosi. Ora, stanca di sedare capricci magici, è partita in cerca di avventure, determinata ad accrescere il suo sapere e a dimostrare che il suo talento va ben oltre il semplice accudimento di piccoli apprendisti indisciplinati.</t>
+  </si>
+  <si>
+    <t>Enea non ricorda il suono del suo nome né il volto della sua famiglia; tutto ciò che possiede è un'armatura ammaccata e una cicatrice profonda che gli attraversa il petto. Risvegliatosi su un campo di battaglia disseminato di cadaveri, ha scoperto che, pur avendo smarrito il passato, i suoi muscoli conservano una memoria letale: ogni fendente, ogni parata e ogni tattica bellica gli tornano naturali come il respiro. Senza radici a cui tornare, ora vaga per i regni come mercenario, cercando tra le pieghe di ogni scontro l'unico nemico capace di svelargli chi fosse prima del fragore delle armi.</t>
+  </si>
+  <si>
+    <t>Celebre tra le nebbie del Lago Brodom per la sua maestria nel navigare acque insidiose, Gabbro non è un avventuriero comune. Questo Bullywug dalla pelle umida impugna un enorme clarinetto di legno stagionato che funge tanto da arma contundente quanto da strumento musicale. In battaglia, la sua musica è un'arma a doppio taglio: una nota stonata può scagliare il nemico a terra, mentre un soffio armonioso è in grado di ritemprare lo spirito dei suoi compagni. Viaggia ora lontano dalle sue paludi natie, convinto che il mondo intero meriti di ascoltare la melodia del Brodom, che sia sotto forma di serenata o di un sonoro colpo in testa.</t>
+  </si>
+  <si>
+    <t>Cresciuto nei vicoli più malfamati della città, Gaspar ha imparato presto che la sopravvivenza dipende dalla capacità di passare inosservati o di diventare qualcun altro. La sua abilità nei furti è leggendaria, ma il suo vero segreto è appeso alla cintura: una testa magica, reliquia di una vecchia avventura, che gli permette di scambiare il proprio volto con quello di una donna misteriosa. Questo artefatto non è solo un travestimento perfetto, ma una parte integrante della sua identità, rendendolo l'infiltrato più sfuggente e camaleontico che le gilde criminali abbiano mai conosciuto.</t>
+  </si>
+  <si>
+    <t>Custode silenzioso del cuore pulsante dei boschi di Dragonlance, Levorax è un dragonide verde che ha dedicato ogni respiro alla protezione della natura. Formatosi sotto l'ala protettrice dell'antico drago verde Veridios, ha appreso che la foresta non è solo un ecosistema, ma un organismo vivente che richiede un equilibrio costante tra crescita e decadenza. Levorax non combatte per la gloria, ma funge da estensione della volontà di Veridios, scagliandosi contro chiunque osi violare la sacralità del verde con la stessa implacabile ferocia delle spine e delle radici profonde.</t>
   </si>
 </sst>
 </file>
@@ -367,7 +376,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -406,6 +415,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -760,7 +775,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="4" customFormat="1" ht="242.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" s="4" customFormat="1" ht="280.5" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>44</v>
       </c>
@@ -782,7 +797,7 @@
         <v>17</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="J2" s="3">
         <v>116</v>
@@ -791,7 +806,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" s="4" customFormat="1" ht="153" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>41</v>
       </c>
@@ -812,7 +827,9 @@
       <c r="H3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="3"/>
+      <c r="I3" s="3" t="s">
+        <v>77</v>
+      </c>
       <c r="J3" s="3">
         <v>47</v>
       </c>
@@ -841,9 +858,7 @@
       <c r="H4" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>65</v>
-      </c>
+      <c r="I4" s="3"/>
       <c r="J4" s="3">
         <v>36</v>
       </c>
@@ -851,7 +866,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" s="4" customFormat="1" ht="195" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>39</v>
       </c>
@@ -872,13 +887,15 @@
       <c r="H5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="3"/>
+      <c r="I5" s="15" t="s">
+        <v>78</v>
+      </c>
       <c r="J5" s="3"/>
       <c r="K5" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:11" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" s="4" customFormat="1" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>20</v>
       </c>
@@ -904,7 +921,7 @@
         <v>17</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>26</v>
@@ -913,7 +930,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" s="4" customFormat="1" ht="153" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>37</v>
       </c>
@@ -934,7 +951,9 @@
       <c r="H7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="3"/>
+      <c r="I7" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J7" s="3"/>
       <c r="K7" s="5" t="s">
         <v>51</v>
@@ -998,7 +1017,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" s="4" customFormat="1" ht="195" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>28</v>
       </c>
@@ -1019,7 +1038,9 @@
       <c r="H10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="3"/>
+      <c r="I10" s="16" t="s">
+        <v>81</v>
+      </c>
       <c r="J10" s="3">
         <v>80</v>
       </c>
@@ -1134,7 +1155,7 @@
     </row>
     <row r="14" spans="1:11" ht="180" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>45</v>
@@ -1143,22 +1164,22 @@
         <v>3</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>23</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G14" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="J14" s="12">
         <v>78</v>
@@ -1169,10 +1190,10 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
@@ -1186,10 +1207,10 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
@@ -1203,7 +1224,7 @@
     </row>
     <row r="17" spans="1:11" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>21</v>
@@ -1212,22 +1233,22 @@
         <v>3</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>23</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="G17" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="J17" s="13">
         <v>10</v>
@@ -1248,25 +1269,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_activity xmlns="b29cbc76-272b-40e5-b4ba-3e4af727d16b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100335EAE044E422D4BAEC0B1BC71186902" ma:contentTypeVersion="20" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="8191542849a603e5cc73d892766c41f0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns3="b29cbc76-272b-40e5-b4ba-3e4af727d16b" xmlns:ns4="abdbd0a1-ed93-4afe-bb88-a490c0734ad3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cc47de22a57756af56b6fd27515aad7d" ns1:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1536,10 +1538,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_activity xmlns="b29cbc76-272b-40e5-b4ba-3e4af727d16b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{702E6FB5-6A67-4034-9986-FD37F4044FFB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E71A66E7-14C5-4436-B338-E9FE6616C4F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="b29cbc76-272b-40e5-b4ba-3e4af727d16b"/>
+    <ds:schemaRef ds:uri="abdbd0a1-ed93-4afe-bb88-a490c0734ad3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1563,21 +1596,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E71A66E7-14C5-4436-B338-E9FE6616C4F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{702E6FB5-6A67-4034-9986-FD37F4044FFB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="b29cbc76-272b-40e5-b4ba-3e4af727d16b"/>
-    <ds:schemaRef ds:uri="abdbd0a1-ed93-4afe-bb88-a490c0734ad3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>